<commit_message>
Extend multi-strategy portfolio risk audit
</commit_message>
<xml_diff>
--- a/templates/private-portfolio-template.xlsx
+++ b/templates/private-portfolio-template.xlsx
@@ -2,12 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Snapshot" sheetId="1" r:id="R67f9ab74c8b24368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="2" r:id="R291c8b51d8d64ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash" sheetId="3" r:id="Rba05502e460f4f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obligations" sheetId="4" r:id="R913f23b5a5af4564"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX" sheetId="5" r:id="R603c51cd58aa4a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="6" r:id="R8d3d124aa6fe4278"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Snapshot" sheetId="1" r:id="R0f326251f9fd4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="2" r:id="R09f2444119b44c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash" sheetId="3" r:id="R341bb23a56034540"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Obligations" sheetId="4" r:id="R9f2c308c1f8e4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX" sheetId="5" r:id="R2f098010fde64390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="6" r:id="R8ce3471e4eda4a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RiskSensitivities" sheetId="7" r:id="R9c45b962800c4e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RiskScenarios" sheetId="8" r:id="Rcf6592dff97b43c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="202" formatCode="0.000000"/>
+    <x:numFmt numFmtId="203" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -63,7 +66,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +76,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -93,7 +101,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -111,6 +119,15 @@
     <x:xf numFmtId="200" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -345,7 +362,7 @@
         <x:v>source_version</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4230,8 +4247,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="83" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -4295,6 +4312,153 @@
         <x:v>No compartir esta hoja ni exportarla a GitHub Pages o al repositorio público.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11" ht="42" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>RiskSensitivities</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="str">
+        <x:v>Una fila por position_id. Usar sensibilidades documentadas; las fracciones de liquidez/default van de 0 a 1. No inventar valores.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="42" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>RiskScenarios</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>Los tres shocks soberanos son fijos (+100/+300/+500 bps). Completar FX, inflación, liquidez ARS y default sólo con parámetros aprobados; celdas vacías producen UNKNOWN.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="36" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="42" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>position_id</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>sovereign_spread_duration_years</x:v>
+      </x:c>
+      <x:c r="C1" s="17" t="str">
+        <x:v>fx_sensitivity_pct_per_100pct_move</x:v>
+      </x:c>
+      <x:c r="D1" s="17" t="str">
+        <x:v>inflation_sensitivity_pct_per_100pct_shock</x:v>
+      </x:c>
+      <x:c r="E1" s="17" t="str">
+        <x:v>ars_liquidity_exposure_fraction</x:v>
+      </x:c>
+      <x:c r="F1" s="17" t="str">
+        <x:v>default_loss_exposure_fraction</x:v>
+      </x:c>
+      <x:c r="G1" s="17" t="str">
+        <x:v>argentina_indirect_exposure_pct</x:v>
+      </x:c>
+      <x:c r="H1" s="17" t="str">
+        <x:v>source_ref</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="17" t="str">
+        <x:v>scenario</x:v>
+      </x:c>
+      <x:c r="B1" s="17" t="str">
+        <x:v>shock_value</x:v>
+      </x:c>
+      <x:c r="C1" s="17" t="str">
+        <x:v>source_ref</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="14" t="str">
+        <x:v>sovereign_spread_100bps</x:v>
+      </x:c>
+      <x:c r="B2" s="18" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str">
+        <x:v>SDD requirements.md REQ-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="14" t="str">
+        <x:v>sovereign_spread_300bps</x:v>
+      </x:c>
+      <x:c r="B3" s="18" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>SDD requirements.md REQ-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="14" t="str">
+        <x:v>sovereign_spread_500bps</x:v>
+      </x:c>
+      <x:c r="B4" s="18" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>SDD requirements.md REQ-18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14" t="str">
+        <x:v>fx_stress</x:v>
+      </x:c>
+      <x:c r="B5" s="18"/>
+      <x:c r="C5" s="14" t="str"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14" t="str">
+        <x:v>extreme_inflation</x:v>
+      </x:c>
+      <x:c r="B6" s="18"/>
+      <x:c r="C6" s="14" t="str"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="14" t="str">
+        <x:v>ars_liquidity</x:v>
+      </x:c>
+      <x:c r="B7" s="18"/>
+      <x:c r="C7" s="14" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14" t="str">
+        <x:v>default_restructuring</x:v>
+      </x:c>
+      <x:c r="B8" s="18"/>
+      <x:c r="C8" s="14" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>